<commit_message>
fix(inpp): alinea metodo de fuente del perfil con el conector.
Corrige config/indicadores_meta.json para que la fuente del INPP
coincida con el método reportado por el conector (INEGI BIE API (INPP)).
Regenera datos, Excel y manifest con la metadata corregida.

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/downloads/indicadores/EMIM/EMIM_datos.xlsx
+++ b/downloads/indicadores/EMIM/EMIM_datos.xlsx
@@ -14712,7 +14712,7 @@
         <v>-0.038393</v>
       </c>
       <c r="E220" s="7" t="n">
-        <v>0.006542</v>
+        <v>0.007</v>
       </c>
       <c r="F220" s="7" t="n">
         <v>0.011</v>
@@ -14727,7 +14727,7 @@
         <v>-0.003941</v>
       </c>
       <c r="J220" s="7" t="n">
-        <v>-0.019399</v>
+        <v>-0.019</v>
       </c>
       <c r="K220" s="7" t="n">
         <v>-0.003</v>
@@ -14742,7 +14742,7 @@
         <v>-0.050048</v>
       </c>
       <c r="O220" s="7" t="n">
-        <v>-0.027586</v>
+        <v>-0.028</v>
       </c>
       <c r="P220" s="7" t="n">
         <v>0.004</v>
@@ -14790,13 +14790,13 @@
         <v>45627</v>
       </c>
       <c r="C221" s="9" t="n">
-        <v>99.2</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="D221" s="10" t="n">
         <v>-0.07892299999999999</v>
       </c>
       <c r="E221" s="10" t="n">
-        <v>-0.004016</v>
+        <v>-0.002</v>
       </c>
       <c r="F221" s="10" t="n">
         <v>-0.015</v>
@@ -14805,13 +14805,13 @@
         <v>0.002</v>
       </c>
       <c r="H221" s="9" t="n">
-        <v>100.3</v>
+        <v>100.4</v>
       </c>
       <c r="I221" s="10" t="n">
         <v>-0.007913</v>
       </c>
       <c r="J221" s="10" t="n">
-        <v>-0.01763</v>
+        <v>-0.017</v>
       </c>
       <c r="K221" s="10" t="n">
         <v>0</v>
@@ -14826,7 +14826,7 @@
         <v>-0.065856</v>
       </c>
       <c r="O221" s="10" t="n">
-        <v>-0.024339</v>
+        <v>-0.024</v>
       </c>
       <c r="P221" s="10" t="n">
         <v>-0.008</v>
@@ -14880,7 +14880,7 @@
         <v>0.082661</v>
       </c>
       <c r="E222" s="7" t="n">
-        <v>-0.012868</v>
+        <v>-0.016</v>
       </c>
       <c r="F222" s="7" t="n">
         <v>-0.004</v>
@@ -14895,7 +14895,7 @@
         <v>0.0009970000000000001</v>
       </c>
       <c r="J222" s="7" t="n">
-        <v>-0.009861999999999999</v>
+        <v>-0.011</v>
       </c>
       <c r="K222" s="7" t="n">
         <v>0.002</v>
@@ -14910,7 +14910,7 @@
         <v>0.074837</v>
       </c>
       <c r="O222" s="7" t="n">
-        <v>-0.008999999999999999</v>
+        <v>-0.01</v>
       </c>
       <c r="P222" s="7" t="n">
         <v>-0.003</v>
@@ -14958,13 +14958,13 @@
         <v>45689</v>
       </c>
       <c r="C223" s="9" t="n">
-        <v>106</v>
+        <v>106.1</v>
       </c>
       <c r="D223" s="10" t="n">
         <v>-0.013035</v>
       </c>
       <c r="E223" s="10" t="n">
-        <v>-0.013953</v>
+        <v>-0.015</v>
       </c>
       <c r="F223" s="10" t="n">
         <v>0.026</v>
@@ -14979,7 +14979,7 @@
         <v>0</v>
       </c>
       <c r="J223" s="10" t="n">
-        <v>-0.011811</v>
+        <v>-0.012</v>
       </c>
       <c r="K223" s="10" t="n">
         <v>-0.003</v>
@@ -14994,7 +14994,7 @@
         <v>-0.058527</v>
       </c>
       <c r="O223" s="10" t="n">
-        <v>-0.045036</v>
+        <v>-0.045</v>
       </c>
       <c r="P223" s="10" t="n">
         <v>0.011</v>
@@ -15042,13 +15042,13 @@
         <v>45717</v>
       </c>
       <c r="C224" s="6" t="n">
-        <v>113.5</v>
+        <v>113.4</v>
       </c>
       <c r="D224" s="7" t="n">
         <v>0.070755</v>
       </c>
       <c r="E224" s="7" t="n">
-        <v>0.020683</v>
+        <v>0.018</v>
       </c>
       <c r="F224" s="7" t="n">
         <v>-0.02</v>
@@ -15063,7 +15063,7 @@
         <v>0.0009959999999999999</v>
       </c>
       <c r="J224" s="7" t="n">
-        <v>-0.008876</v>
+        <v>-0.008999999999999999</v>
       </c>
       <c r="K224" s="7" t="n">
         <v>-0.001</v>
@@ -15072,13 +15072,13 @@
         <v>-0.008</v>
       </c>
       <c r="M224" s="6" t="n">
-        <v>98.3</v>
+        <v>98.2</v>
       </c>
       <c r="N224" s="7" t="n">
         <v>0.053591</v>
       </c>
       <c r="O224" s="7" t="n">
-        <v>0.007172</v>
+        <v>0.006</v>
       </c>
       <c r="P224" s="7" t="n">
         <v>-0.007</v>
@@ -15126,13 +15126,13 @@
         <v>45748</v>
       </c>
       <c r="C225" s="9" t="n">
-        <v>108.9</v>
+        <v>109</v>
       </c>
       <c r="D225" s="10" t="n">
         <v>-0.040529</v>
       </c>
       <c r="E225" s="10" t="n">
-        <v>-0.037986</v>
+        <v>-0.037</v>
       </c>
       <c r="F225" s="10" t="n">
         <v>-0.001</v>
@@ -15141,13 +15141,13 @@
         <v>-0.008999999999999999</v>
       </c>
       <c r="H225" s="9" t="n">
-        <v>100.5</v>
+        <v>100.4</v>
       </c>
       <c r="I225" s="10" t="n">
         <v>0</v>
       </c>
       <c r="J225" s="10" t="n">
-        <v>-0.015671</v>
+        <v>-0.016</v>
       </c>
       <c r="K225" s="10" t="n">
         <v>-0.004</v>
@@ -15156,13 +15156,13 @@
         <v>-0.016</v>
       </c>
       <c r="M225" s="9" t="n">
-        <v>97.40000000000001</v>
+        <v>97.3</v>
       </c>
       <c r="N225" s="10" t="n">
         <v>-0.009155999999999999</v>
       </c>
       <c r="O225" s="10" t="n">
-        <v>-0.032771</v>
+        <v>-0.034</v>
       </c>
       <c r="P225" s="10" t="n">
         <v>0.005</v>
@@ -15210,13 +15210,13 @@
         <v>45778</v>
       </c>
       <c r="C226" s="6" t="n">
-        <v>112.1</v>
+        <v>112</v>
       </c>
       <c r="D226" s="7" t="n">
         <v>0.029385</v>
       </c>
       <c r="E226" s="7" t="n">
-        <v>0.005381</v>
+        <v>0.003</v>
       </c>
       <c r="F226" s="7" t="n">
         <v>0.01</v>
@@ -15225,13 +15225,13 @@
         <v>0.01</v>
       </c>
       <c r="H226" s="6" t="n">
-        <v>100.4</v>
+        <v>100.3</v>
       </c>
       <c r="I226" s="7" t="n">
         <v>-0.000995</v>
       </c>
       <c r="J226" s="7" t="n">
-        <v>-0.019531</v>
+        <v>-0.02</v>
       </c>
       <c r="K226" s="7" t="n">
         <v>-0.003</v>
@@ -15246,7 +15246,7 @@
         <v>0.025667</v>
       </c>
       <c r="O226" s="7" t="n">
-        <v>-0.032914</v>
+        <v>-0.033</v>
       </c>
       <c r="P226" s="7" t="n">
         <v>-0.01</v>
@@ -15294,13 +15294,13 @@
         <v>45809</v>
       </c>
       <c r="C227" s="9" t="n">
-        <v>111.9</v>
+        <v>111.8</v>
       </c>
       <c r="D227" s="10" t="n">
         <v>-0.001784</v>
       </c>
       <c r="E227" s="10" t="n">
-        <v>0.031336</v>
+        <v>0.029</v>
       </c>
       <c r="F227" s="10" t="n">
         <v>0.016</v>
@@ -15309,13 +15309,13 @@
         <v>0.023</v>
       </c>
       <c r="H227" s="9" t="n">
-        <v>100.1</v>
+        <v>100</v>
       </c>
       <c r="I227" s="10" t="n">
         <v>-0.002988</v>
       </c>
       <c r="J227" s="10" t="n">
-        <v>-0.019589</v>
+        <v>-0.02</v>
       </c>
       <c r="K227" s="10" t="n">
         <v>-0.002</v>
@@ -15324,13 +15324,13 @@
         <v>-0.02</v>
       </c>
       <c r="M227" s="9" t="n">
-        <v>97.90000000000001</v>
+        <v>97.8</v>
       </c>
       <c r="N227" s="10" t="n">
         <v>-0.02002</v>
       </c>
       <c r="O227" s="10" t="n">
-        <v>-0.013105</v>
+        <v>-0.015</v>
       </c>
       <c r="P227" s="10" t="n">
         <v>0</v>
@@ -15378,13 +15378,13 @@
         <v>45839</v>
       </c>
       <c r="C228" s="6" t="n">
-        <v>110.2</v>
+        <v>110.1</v>
       </c>
       <c r="D228" s="7" t="n">
         <v>-0.015192</v>
       </c>
       <c r="E228" s="7" t="n">
-        <v>-0.000907</v>
+        <v>-0.004</v>
       </c>
       <c r="F228" s="7" t="n">
         <v>-0.027</v>
@@ -15399,7 +15399,7 @@
         <v>-0.003996</v>
       </c>
       <c r="J228" s="7" t="n">
-        <v>-0.022549</v>
+        <v>-0.023</v>
       </c>
       <c r="K228" s="7" t="n">
         <v>-0.002</v>
@@ -15408,13 +15408,13 @@
         <v>-0.023</v>
       </c>
       <c r="M228" s="6" t="n">
-        <v>101.4</v>
+        <v>101.3</v>
       </c>
       <c r="N228" s="7" t="n">
         <v>0.035751</v>
       </c>
       <c r="O228" s="7" t="n">
-        <v>-0.010732</v>
+        <v>-0.012</v>
       </c>
       <c r="P228" s="7" t="n">
         <v>-0.002</v>
@@ -15468,7 +15468,7 @@
         <v>-0.00726</v>
       </c>
       <c r="E229" s="10" t="n">
-        <v>-0.030142</v>
+        <v>-0.03</v>
       </c>
       <c r="F229" s="10" t="n">
         <v>-0.003</v>
@@ -15483,7 +15483,7 @@
         <v>-0.005015</v>
       </c>
       <c r="J229" s="10" t="n">
-        <v>-0.026497</v>
+        <v>-0.026</v>
       </c>
       <c r="K229" s="10" t="n">
         <v>-0.005</v>
@@ -15498,7 +15498,7 @@
         <v>-0.027613</v>
       </c>
       <c r="O229" s="10" t="n">
-        <v>-0.052834</v>
+        <v>-0.053</v>
       </c>
       <c r="P229" s="10" t="n">
         <v>-0.006</v>
@@ -15552,7 +15552,7 @@
         <v>-0.002742</v>
       </c>
       <c r="E230" s="7" t="n">
-        <v>-0.007279</v>
+        <v>-0.007</v>
       </c>
       <c r="F230" s="7" t="n">
         <v>0.002</v>
@@ -15567,7 +15567,7 @@
         <v>-0.001008</v>
       </c>
       <c r="J230" s="7" t="n">
-        <v>-0.025565</v>
+        <v>-0.026</v>
       </c>
       <c r="K230" s="7" t="n">
         <v>-0.001</v>
@@ -15582,7 +15582,7 @@
         <v>-0.017241</v>
       </c>
       <c r="O230" s="7" t="n">
-        <v>-0.018237</v>
+        <v>-0.018</v>
       </c>
       <c r="P230" s="7" t="n">
         <v>-0.004</v>
@@ -15636,7 +15636,7 @@
         <v>0.03483</v>
       </c>
       <c r="E231" s="10" t="n">
-        <v>0.008036</v>
+        <v>0.008</v>
       </c>
       <c r="F231" s="10" t="n">
         <v>0.003</v>
@@ -15651,7 +15651,7 @@
         <v>-0.001009</v>
       </c>
       <c r="J231" s="10" t="n">
-        <v>-0.024631</v>
+        <v>-0.025</v>
       </c>
       <c r="K231" s="10" t="n">
         <v>-0.001</v>
@@ -15666,7 +15666,7 @@
         <v>0.05676</v>
       </c>
       <c r="O231" s="10" t="n">
-        <v>-0.014437</v>
+        <v>-0.014</v>
       </c>
       <c r="P231" s="10" t="n">
         <v>0.006</v>
@@ -15720,7 +15720,7 @@
         <v>-0.045173</v>
       </c>
       <c r="E232" s="7" t="n">
-        <v>0.000929</v>
+        <v>0.001</v>
       </c>
       <c r="F232" s="7" t="n">
         <v>0.01</v>
@@ -15735,7 +15735,7 @@
         <v>-0.007071</v>
       </c>
       <c r="J232" s="7" t="n">
-        <v>-0.027695</v>
+        <v>-0.028</v>
       </c>
       <c r="K232" s="7" t="n">
         <v>-0.004</v>
@@ -15750,7 +15750,7 @@
         <v>-0.080078</v>
       </c>
       <c r="O232" s="7" t="n">
-        <v>-0.045593</v>
+        <v>-0.046</v>
       </c>
       <c r="P232" s="7" t="n">
         <v>-0.006</v>
@@ -15804,7 +15804,7 @@
         <v>-0.039889</v>
       </c>
       <c r="E233" s="10" t="n">
-        <v>0.043347</v>
+        <v>0.043</v>
       </c>
       <c r="F233" s="10" t="n">
         <v>-0.001</v>
@@ -15819,7 +15819,7 @@
         <v>-0.006104</v>
       </c>
       <c r="J233" s="10" t="n">
-        <v>-0.025922</v>
+        <v>-0.026</v>
       </c>
       <c r="K233" s="10" t="n">
         <v>0</v>
@@ -15834,7 +15834,7 @@
         <v>-0.030786</v>
       </c>
       <c r="O233" s="10" t="n">
-        <v>-0.009761000000000001</v>
+        <v>-0.01</v>
       </c>
       <c r="P233" s="10" t="n">
         <v>-0.001</v>
@@ -15888,7 +15888,7 @@
         <v>0.022222</v>
       </c>
       <c r="E234" s="7" t="n">
-        <v>-0.014898</v>
+        <v>-0.015</v>
       </c>
       <c r="F234" s="7" t="n">
         <v>-0.018</v>
@@ -15903,7 +15903,7 @@
         <v>0.002047</v>
       </c>
       <c r="J234" s="7" t="n">
-        <v>-0.0249</v>
+        <v>-0.025</v>
       </c>
       <c r="K234" s="7" t="n">
         <v>0.002</v>
@@ -15918,7 +15918,7 @@
         <v>0.048193</v>
       </c>
       <c r="O234" s="7" t="n">
-        <v>-0.034309</v>
+        <v>-0.034</v>
       </c>
       <c r="P234" s="7" t="n">
         <v>-0.004</v>
@@ -15972,7 +15972,7 @@
         <v>0.012287</v>
       </c>
       <c r="E235" s="10" t="n">
-        <v>0.010377</v>
+        <v>0.01</v>
       </c>
       <c r="F235" s="10" t="n">
         <v>0.034</v>
@@ -15987,7 +15987,7 @@
         <v>-0.001021</v>
       </c>
       <c r="J235" s="10" t="n">
-        <v>-0.025896</v>
+        <v>-0.026</v>
       </c>
       <c r="K235" s="10" t="n">
         <v>-0.003</v>
@@ -16002,7 +16002,7 @@
         <v>-0.055381</v>
       </c>
       <c r="O235" s="10" t="n">
-        <v>-0.031083</v>
+        <v>-0.031</v>
       </c>
       <c r="P235" s="10" t="n">
         <v>0.002</v>
@@ -16056,7 +16056,7 @@
         <v>0.077498</v>
       </c>
       <c r="E236" s="7" t="n">
-        <v>0.01674</v>
+        <v>0.017</v>
       </c>
       <c r="F236" s="7" t="n">
         <v>-0.011</v>
@@ -16071,7 +16071,7 @@
         <v>0.002045</v>
       </c>
       <c r="J236" s="7" t="n">
-        <v>-0.024876</v>
+        <v>-0.025</v>
       </c>
       <c r="K236" s="7" t="n">
         <v>-0.001</v>
@@ -16086,7 +16086,7 @@
         <v>0.06858400000000001</v>
       </c>
       <c r="O236" s="7" t="n">
-        <v>-0.017294</v>
+        <v>-0.017</v>
       </c>
       <c r="P236" s="7" t="n">
         <v>0</v>
@@ -16140,7 +16140,7 @@
         <v>-0.036395</v>
       </c>
       <c r="E237" s="10" t="n">
-        <v>0.02112</v>
+        <v>0.021</v>
       </c>
       <c r="F237" s="10" t="n">
         <v>0.005</v>
@@ -16155,7 +16155,7 @@
         <v>0.00102</v>
       </c>
       <c r="J237" s="10" t="n">
-        <v>-0.023881</v>
+        <v>-0.024</v>
       </c>
       <c r="K237" s="10" t="n">
         <v>-0.002</v>
@@ -16170,7 +16170,7 @@
         <v>0</v>
       </c>
       <c r="O237" s="10" t="n">
-        <v>-0.008214000000000001</v>
+        <v>-0.008</v>
       </c>
       <c r="P237" s="10" t="n">
         <v>0.006</v>
@@ -16224,7 +16224,7 @@
         <v>-0.007194</v>
       </c>
       <c r="E238" s="7" t="n">
-        <v>-0.015165</v>
+        <v>-0.015</v>
       </c>
       <c r="F238" s="7" t="n">
         <v>-0.006</v>
@@ -16239,7 +16239,7 @@
         <v>0.002039</v>
       </c>
       <c r="J238" s="7" t="n">
-        <v>-0.020916</v>
+        <v>-0.021</v>
       </c>
       <c r="K238" s="7" t="n">
         <v>-0.001</v>
@@ -16254,7 +16254,7 @@
         <v>-0.006211</v>
       </c>
       <c r="O238" s="7" t="n">
-        <v>-0.039039</v>
+        <v>-0.039</v>
       </c>
       <c r="P238" s="7" t="n">
         <v>-0.005</v>
@@ -16308,7 +16308,7 @@
         <v>0.002717</v>
       </c>
       <c r="E239" s="10" t="n">
-        <v>-0.010724</v>
+        <v>-0.011</v>
       </c>
       <c r="F239" s="10" t="n">
         <v>0.001</v>
@@ -16323,7 +16323,7 @@
         <v>0.003052</v>
       </c>
       <c r="J239" s="10" t="n">
-        <v>-0.014985</v>
+        <v>-0.015</v>
       </c>
       <c r="K239" s="10" t="n">
         <v>0.001</v>
@@ -16338,7 +16338,7 @@
         <v>0.01875</v>
       </c>
       <c r="O239" s="10" t="n">
-        <v>-0.001021</v>
+        <v>-0.001</v>
       </c>
       <c r="P239" s="10" t="n">
         <v>0.001</v>

</xml_diff>

<commit_message>
data: restaura datos saludables desde aa717e1 y regenera offline.
Corrige los estados ERROR DE FUENTE causados por errores transitorios de
DNS en la última ejecución online. Restaura los datos limpios del primer
commit del feature INPP, aplica la metadata corregida del perfil y
regenera offline datos, Excel y resumen con todos los indicadores ACTUALIZADO.

- build_data --offline, build_excel, validate y pytest pasan.
- 113 tests passed, 0 errores críticos.

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/downloads/indicadores/EMIM/EMIM_datos.xlsx
+++ b/downloads/indicadores/EMIM/EMIM_datos.xlsx
@@ -14712,7 +14712,7 @@
         <v>-0.038393</v>
       </c>
       <c r="E220" s="7" t="n">
-        <v>0.007</v>
+        <v>0.006542</v>
       </c>
       <c r="F220" s="7" t="n">
         <v>0.011</v>
@@ -14727,7 +14727,7 @@
         <v>-0.003941</v>
       </c>
       <c r="J220" s="7" t="n">
-        <v>-0.019</v>
+        <v>-0.019399</v>
       </c>
       <c r="K220" s="7" t="n">
         <v>-0.003</v>
@@ -14742,7 +14742,7 @@
         <v>-0.050048</v>
       </c>
       <c r="O220" s="7" t="n">
-        <v>-0.028</v>
+        <v>-0.027586</v>
       </c>
       <c r="P220" s="7" t="n">
         <v>0.004</v>
@@ -14790,13 +14790,13 @@
         <v>45627</v>
       </c>
       <c r="C221" s="9" t="n">
-        <v>99.40000000000001</v>
+        <v>99.2</v>
       </c>
       <c r="D221" s="10" t="n">
         <v>-0.07892299999999999</v>
       </c>
       <c r="E221" s="10" t="n">
-        <v>-0.002</v>
+        <v>-0.004016</v>
       </c>
       <c r="F221" s="10" t="n">
         <v>-0.015</v>
@@ -14805,13 +14805,13 @@
         <v>0.002</v>
       </c>
       <c r="H221" s="9" t="n">
-        <v>100.4</v>
+        <v>100.3</v>
       </c>
       <c r="I221" s="10" t="n">
         <v>-0.007913</v>
       </c>
       <c r="J221" s="10" t="n">
-        <v>-0.017</v>
+        <v>-0.01763</v>
       </c>
       <c r="K221" s="10" t="n">
         <v>0</v>
@@ -14826,7 +14826,7 @@
         <v>-0.065856</v>
       </c>
       <c r="O221" s="10" t="n">
-        <v>-0.024</v>
+        <v>-0.024339</v>
       </c>
       <c r="P221" s="10" t="n">
         <v>-0.008</v>
@@ -14880,7 +14880,7 @@
         <v>0.082661</v>
       </c>
       <c r="E222" s="7" t="n">
-        <v>-0.016</v>
+        <v>-0.012868</v>
       </c>
       <c r="F222" s="7" t="n">
         <v>-0.004</v>
@@ -14895,7 +14895,7 @@
         <v>0.0009970000000000001</v>
       </c>
       <c r="J222" s="7" t="n">
-        <v>-0.011</v>
+        <v>-0.009861999999999999</v>
       </c>
       <c r="K222" s="7" t="n">
         <v>0.002</v>
@@ -14910,7 +14910,7 @@
         <v>0.074837</v>
       </c>
       <c r="O222" s="7" t="n">
-        <v>-0.01</v>
+        <v>-0.008999999999999999</v>
       </c>
       <c r="P222" s="7" t="n">
         <v>-0.003</v>
@@ -14958,13 +14958,13 @@
         <v>45689</v>
       </c>
       <c r="C223" s="9" t="n">
-        <v>106.1</v>
+        <v>106</v>
       </c>
       <c r="D223" s="10" t="n">
         <v>-0.013035</v>
       </c>
       <c r="E223" s="10" t="n">
-        <v>-0.015</v>
+        <v>-0.013953</v>
       </c>
       <c r="F223" s="10" t="n">
         <v>0.026</v>
@@ -14979,7 +14979,7 @@
         <v>0</v>
       </c>
       <c r="J223" s="10" t="n">
-        <v>-0.012</v>
+        <v>-0.011811</v>
       </c>
       <c r="K223" s="10" t="n">
         <v>-0.003</v>
@@ -14994,7 +14994,7 @@
         <v>-0.058527</v>
       </c>
       <c r="O223" s="10" t="n">
-        <v>-0.045</v>
+        <v>-0.045036</v>
       </c>
       <c r="P223" s="10" t="n">
         <v>0.011</v>
@@ -15042,13 +15042,13 @@
         <v>45717</v>
       </c>
       <c r="C224" s="6" t="n">
-        <v>113.4</v>
+        <v>113.5</v>
       </c>
       <c r="D224" s="7" t="n">
         <v>0.070755</v>
       </c>
       <c r="E224" s="7" t="n">
-        <v>0.018</v>
+        <v>0.020683</v>
       </c>
       <c r="F224" s="7" t="n">
         <v>-0.02</v>
@@ -15063,7 +15063,7 @@
         <v>0.0009959999999999999</v>
       </c>
       <c r="J224" s="7" t="n">
-        <v>-0.008999999999999999</v>
+        <v>-0.008876</v>
       </c>
       <c r="K224" s="7" t="n">
         <v>-0.001</v>
@@ -15072,13 +15072,13 @@
         <v>-0.008</v>
       </c>
       <c r="M224" s="6" t="n">
-        <v>98.2</v>
+        <v>98.3</v>
       </c>
       <c r="N224" s="7" t="n">
         <v>0.053591</v>
       </c>
       <c r="O224" s="7" t="n">
-        <v>0.006</v>
+        <v>0.007172</v>
       </c>
       <c r="P224" s="7" t="n">
         <v>-0.007</v>
@@ -15126,13 +15126,13 @@
         <v>45748</v>
       </c>
       <c r="C225" s="9" t="n">
-        <v>109</v>
+        <v>108.9</v>
       </c>
       <c r="D225" s="10" t="n">
         <v>-0.040529</v>
       </c>
       <c r="E225" s="10" t="n">
-        <v>-0.037</v>
+        <v>-0.037986</v>
       </c>
       <c r="F225" s="10" t="n">
         <v>-0.001</v>
@@ -15141,13 +15141,13 @@
         <v>-0.008999999999999999</v>
       </c>
       <c r="H225" s="9" t="n">
-        <v>100.4</v>
+        <v>100.5</v>
       </c>
       <c r="I225" s="10" t="n">
         <v>0</v>
       </c>
       <c r="J225" s="10" t="n">
-        <v>-0.016</v>
+        <v>-0.015671</v>
       </c>
       <c r="K225" s="10" t="n">
         <v>-0.004</v>
@@ -15156,13 +15156,13 @@
         <v>-0.016</v>
       </c>
       <c r="M225" s="9" t="n">
-        <v>97.3</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="N225" s="10" t="n">
         <v>-0.009155999999999999</v>
       </c>
       <c r="O225" s="10" t="n">
-        <v>-0.034</v>
+        <v>-0.032771</v>
       </c>
       <c r="P225" s="10" t="n">
         <v>0.005</v>
@@ -15210,13 +15210,13 @@
         <v>45778</v>
       </c>
       <c r="C226" s="6" t="n">
-        <v>112</v>
+        <v>112.1</v>
       </c>
       <c r="D226" s="7" t="n">
         <v>0.029385</v>
       </c>
       <c r="E226" s="7" t="n">
-        <v>0.003</v>
+        <v>0.005381</v>
       </c>
       <c r="F226" s="7" t="n">
         <v>0.01</v>
@@ -15225,13 +15225,13 @@
         <v>0.01</v>
       </c>
       <c r="H226" s="6" t="n">
-        <v>100.3</v>
+        <v>100.4</v>
       </c>
       <c r="I226" s="7" t="n">
         <v>-0.000995</v>
       </c>
       <c r="J226" s="7" t="n">
-        <v>-0.02</v>
+        <v>-0.019531</v>
       </c>
       <c r="K226" s="7" t="n">
         <v>-0.003</v>
@@ -15246,7 +15246,7 @@
         <v>0.025667</v>
       </c>
       <c r="O226" s="7" t="n">
-        <v>-0.033</v>
+        <v>-0.032914</v>
       </c>
       <c r="P226" s="7" t="n">
         <v>-0.01</v>
@@ -15294,13 +15294,13 @@
         <v>45809</v>
       </c>
       <c r="C227" s="9" t="n">
-        <v>111.8</v>
+        <v>111.9</v>
       </c>
       <c r="D227" s="10" t="n">
         <v>-0.001784</v>
       </c>
       <c r="E227" s="10" t="n">
-        <v>0.029</v>
+        <v>0.031336</v>
       </c>
       <c r="F227" s="10" t="n">
         <v>0.016</v>
@@ -15309,13 +15309,13 @@
         <v>0.023</v>
       </c>
       <c r="H227" s="9" t="n">
-        <v>100</v>
+        <v>100.1</v>
       </c>
       <c r="I227" s="10" t="n">
         <v>-0.002988</v>
       </c>
       <c r="J227" s="10" t="n">
-        <v>-0.02</v>
+        <v>-0.019589</v>
       </c>
       <c r="K227" s="10" t="n">
         <v>-0.002</v>
@@ -15324,13 +15324,13 @@
         <v>-0.02</v>
       </c>
       <c r="M227" s="9" t="n">
-        <v>97.8</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="N227" s="10" t="n">
         <v>-0.02002</v>
       </c>
       <c r="O227" s="10" t="n">
-        <v>-0.015</v>
+        <v>-0.013105</v>
       </c>
       <c r="P227" s="10" t="n">
         <v>0</v>
@@ -15378,13 +15378,13 @@
         <v>45839</v>
       </c>
       <c r="C228" s="6" t="n">
-        <v>110.1</v>
+        <v>110.2</v>
       </c>
       <c r="D228" s="7" t="n">
         <v>-0.015192</v>
       </c>
       <c r="E228" s="7" t="n">
-        <v>-0.004</v>
+        <v>-0.000907</v>
       </c>
       <c r="F228" s="7" t="n">
         <v>-0.027</v>
@@ -15399,7 +15399,7 @@
         <v>-0.003996</v>
       </c>
       <c r="J228" s="7" t="n">
-        <v>-0.023</v>
+        <v>-0.022549</v>
       </c>
       <c r="K228" s="7" t="n">
         <v>-0.002</v>
@@ -15408,13 +15408,13 @@
         <v>-0.023</v>
       </c>
       <c r="M228" s="6" t="n">
-        <v>101.3</v>
+        <v>101.4</v>
       </c>
       <c r="N228" s="7" t="n">
         <v>0.035751</v>
       </c>
       <c r="O228" s="7" t="n">
-        <v>-0.012</v>
+        <v>-0.010732</v>
       </c>
       <c r="P228" s="7" t="n">
         <v>-0.002</v>
@@ -15468,7 +15468,7 @@
         <v>-0.00726</v>
       </c>
       <c r="E229" s="10" t="n">
-        <v>-0.03</v>
+        <v>-0.030142</v>
       </c>
       <c r="F229" s="10" t="n">
         <v>-0.003</v>
@@ -15483,7 +15483,7 @@
         <v>-0.005015</v>
       </c>
       <c r="J229" s="10" t="n">
-        <v>-0.026</v>
+        <v>-0.026497</v>
       </c>
       <c r="K229" s="10" t="n">
         <v>-0.005</v>
@@ -15498,7 +15498,7 @@
         <v>-0.027613</v>
       </c>
       <c r="O229" s="10" t="n">
-        <v>-0.053</v>
+        <v>-0.052834</v>
       </c>
       <c r="P229" s="10" t="n">
         <v>-0.006</v>
@@ -15552,7 +15552,7 @@
         <v>-0.002742</v>
       </c>
       <c r="E230" s="7" t="n">
-        <v>-0.007</v>
+        <v>-0.007279</v>
       </c>
       <c r="F230" s="7" t="n">
         <v>0.002</v>
@@ -15567,7 +15567,7 @@
         <v>-0.001008</v>
       </c>
       <c r="J230" s="7" t="n">
-        <v>-0.026</v>
+        <v>-0.025565</v>
       </c>
       <c r="K230" s="7" t="n">
         <v>-0.001</v>
@@ -15582,7 +15582,7 @@
         <v>-0.017241</v>
       </c>
       <c r="O230" s="7" t="n">
-        <v>-0.018</v>
+        <v>-0.018237</v>
       </c>
       <c r="P230" s="7" t="n">
         <v>-0.004</v>
@@ -15636,7 +15636,7 @@
         <v>0.03483</v>
       </c>
       <c r="E231" s="10" t="n">
-        <v>0.008</v>
+        <v>0.008036</v>
       </c>
       <c r="F231" s="10" t="n">
         <v>0.003</v>
@@ -15651,7 +15651,7 @@
         <v>-0.001009</v>
       </c>
       <c r="J231" s="10" t="n">
-        <v>-0.025</v>
+        <v>-0.024631</v>
       </c>
       <c r="K231" s="10" t="n">
         <v>-0.001</v>
@@ -15666,7 +15666,7 @@
         <v>0.05676</v>
       </c>
       <c r="O231" s="10" t="n">
-        <v>-0.014</v>
+        <v>-0.014437</v>
       </c>
       <c r="P231" s="10" t="n">
         <v>0.006</v>
@@ -15720,7 +15720,7 @@
         <v>-0.045173</v>
       </c>
       <c r="E232" s="7" t="n">
-        <v>0.001</v>
+        <v>0.000929</v>
       </c>
       <c r="F232" s="7" t="n">
         <v>0.01</v>
@@ -15735,7 +15735,7 @@
         <v>-0.007071</v>
       </c>
       <c r="J232" s="7" t="n">
-        <v>-0.028</v>
+        <v>-0.027695</v>
       </c>
       <c r="K232" s="7" t="n">
         <v>-0.004</v>
@@ -15750,7 +15750,7 @@
         <v>-0.080078</v>
       </c>
       <c r="O232" s="7" t="n">
-        <v>-0.046</v>
+        <v>-0.045593</v>
       </c>
       <c r="P232" s="7" t="n">
         <v>-0.006</v>
@@ -15804,7 +15804,7 @@
         <v>-0.039889</v>
       </c>
       <c r="E233" s="10" t="n">
-        <v>0.043</v>
+        <v>0.043347</v>
       </c>
       <c r="F233" s="10" t="n">
         <v>-0.001</v>
@@ -15819,7 +15819,7 @@
         <v>-0.006104</v>
       </c>
       <c r="J233" s="10" t="n">
-        <v>-0.026</v>
+        <v>-0.025922</v>
       </c>
       <c r="K233" s="10" t="n">
         <v>0</v>
@@ -15834,7 +15834,7 @@
         <v>-0.030786</v>
       </c>
       <c r="O233" s="10" t="n">
-        <v>-0.01</v>
+        <v>-0.009761000000000001</v>
       </c>
       <c r="P233" s="10" t="n">
         <v>-0.001</v>
@@ -15888,7 +15888,7 @@
         <v>0.022222</v>
       </c>
       <c r="E234" s="7" t="n">
-        <v>-0.015</v>
+        <v>-0.014898</v>
       </c>
       <c r="F234" s="7" t="n">
         <v>-0.018</v>
@@ -15903,7 +15903,7 @@
         <v>0.002047</v>
       </c>
       <c r="J234" s="7" t="n">
-        <v>-0.025</v>
+        <v>-0.0249</v>
       </c>
       <c r="K234" s="7" t="n">
         <v>0.002</v>
@@ -15918,7 +15918,7 @@
         <v>0.048193</v>
       </c>
       <c r="O234" s="7" t="n">
-        <v>-0.034</v>
+        <v>-0.034309</v>
       </c>
       <c r="P234" s="7" t="n">
         <v>-0.004</v>
@@ -15972,7 +15972,7 @@
         <v>0.012287</v>
       </c>
       <c r="E235" s="10" t="n">
-        <v>0.01</v>
+        <v>0.010377</v>
       </c>
       <c r="F235" s="10" t="n">
         <v>0.034</v>
@@ -15987,7 +15987,7 @@
         <v>-0.001021</v>
       </c>
       <c r="J235" s="10" t="n">
-        <v>-0.026</v>
+        <v>-0.025896</v>
       </c>
       <c r="K235" s="10" t="n">
         <v>-0.003</v>
@@ -16002,7 +16002,7 @@
         <v>-0.055381</v>
       </c>
       <c r="O235" s="10" t="n">
-        <v>-0.031</v>
+        <v>-0.031083</v>
       </c>
       <c r="P235" s="10" t="n">
         <v>0.002</v>
@@ -16056,7 +16056,7 @@
         <v>0.077498</v>
       </c>
       <c r="E236" s="7" t="n">
-        <v>0.017</v>
+        <v>0.01674</v>
       </c>
       <c r="F236" s="7" t="n">
         <v>-0.011</v>
@@ -16071,7 +16071,7 @@
         <v>0.002045</v>
       </c>
       <c r="J236" s="7" t="n">
-        <v>-0.025</v>
+        <v>-0.024876</v>
       </c>
       <c r="K236" s="7" t="n">
         <v>-0.001</v>
@@ -16086,7 +16086,7 @@
         <v>0.06858400000000001</v>
       </c>
       <c r="O236" s="7" t="n">
-        <v>-0.017</v>
+        <v>-0.017294</v>
       </c>
       <c r="P236" s="7" t="n">
         <v>0</v>
@@ -16140,7 +16140,7 @@
         <v>-0.036395</v>
       </c>
       <c r="E237" s="10" t="n">
-        <v>0.021</v>
+        <v>0.02112</v>
       </c>
       <c r="F237" s="10" t="n">
         <v>0.005</v>
@@ -16155,7 +16155,7 @@
         <v>0.00102</v>
       </c>
       <c r="J237" s="10" t="n">
-        <v>-0.024</v>
+        <v>-0.023881</v>
       </c>
       <c r="K237" s="10" t="n">
         <v>-0.002</v>
@@ -16170,7 +16170,7 @@
         <v>0</v>
       </c>
       <c r="O237" s="10" t="n">
-        <v>-0.008</v>
+        <v>-0.008214000000000001</v>
       </c>
       <c r="P237" s="10" t="n">
         <v>0.006</v>
@@ -16224,7 +16224,7 @@
         <v>-0.007194</v>
       </c>
       <c r="E238" s="7" t="n">
-        <v>-0.015</v>
+        <v>-0.015165</v>
       </c>
       <c r="F238" s="7" t="n">
         <v>-0.006</v>
@@ -16239,7 +16239,7 @@
         <v>0.002039</v>
       </c>
       <c r="J238" s="7" t="n">
-        <v>-0.021</v>
+        <v>-0.020916</v>
       </c>
       <c r="K238" s="7" t="n">
         <v>-0.001</v>
@@ -16254,7 +16254,7 @@
         <v>-0.006211</v>
       </c>
       <c r="O238" s="7" t="n">
-        <v>-0.039</v>
+        <v>-0.039039</v>
       </c>
       <c r="P238" s="7" t="n">
         <v>-0.005</v>
@@ -16308,7 +16308,7 @@
         <v>0.002717</v>
       </c>
       <c r="E239" s="10" t="n">
-        <v>-0.011</v>
+        <v>-0.010724</v>
       </c>
       <c r="F239" s="10" t="n">
         <v>0.001</v>
@@ -16323,7 +16323,7 @@
         <v>0.003052</v>
       </c>
       <c r="J239" s="10" t="n">
-        <v>-0.015</v>
+        <v>-0.014985</v>
       </c>
       <c r="K239" s="10" t="n">
         <v>0.001</v>
@@ -16338,7 +16338,7 @@
         <v>0.01875</v>
       </c>
       <c r="O239" s="10" t="n">
-        <v>-0.001</v>
+        <v>-0.001021</v>
       </c>
       <c r="P239" s="10" t="n">
         <v>0.001</v>

</xml_diff>